<commit_message>
Replace example data with user's actual budget and add Konton sheet
Replaces the placeholder rows in Inkomst, Utgifter and Sparmål with the
user's real numbers (lön efter skatt 27 840 kr, recurring expenses incl.
hyra, mat, fordon, försäkringar, prenumerationer; savings goals Buffert
60 000 kr and Snöskoter 40 000 kr). Adds a new Konton sheet tracking
Sparkonto (34 000 kr) and Allkonto (2 600 kr) plus a "Saldo på konton"
KPI on the dashboard. Yearly costs (bilskatt, bilförsäkring) are split
into monthly averages.

https://claude.ai/code/session_01TGDrghwEeC6PfsKqYZFCU5
</commit_message>
<xml_diff>
--- a/Monthly_Budget_SEK.xlsx
+++ b/Monthly_Budget_SEK.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Inkomst" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Utgifter" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Sparmål" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Konton" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="Kategorier">Inställningar!$A$2:$A$11</definedName>
@@ -855,25 +856,25 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>Inkomst!C7</f>
+        <f>Inkomst!C4</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Total utgift</t>
+          <t>Total utgift (budget)</t>
         </is>
       </c>
       <c r="B6" s="5">
-        <f>SUM(Utgifter!E2:E61)</f>
+        <f>SUM(Utgifter!D2:D61)</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Netto / Sparat</t>
+          <t>Netto enligt budget</t>
         </is>
       </c>
       <c r="B7" s="5">
@@ -895,11 +896,22 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Budget kvar</t>
+          <t>Faktiskt utgift hittills</t>
         </is>
       </c>
       <c r="B9" s="5">
-        <f>SUM(Utgifter!D2:D61)-SUM(Utgifter!E2:E61)</f>
+        <f>SUM(Utgifter!E2:E61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Saldo på konton</t>
+        </is>
+      </c>
+      <c r="B10" s="5">
+        <f>Konton!B4</f>
         <v/>
       </c>
     </row>
@@ -1290,7 +1302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1324,14 +1336,14 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Lön</t>
+          <t>Lön efter skatt</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>35000</v>
+        <v>27840</v>
       </c>
       <c r="C2" s="10" t="n">
-        <v>0</v>
+        <v>27840</v>
       </c>
       <c r="D2" s="10">
         <f>C2-B2</f>
@@ -1341,7 +1353,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Bonus</t>
+          <t>Övrig inkomst</t>
         </is>
       </c>
       <c r="B3" s="10" t="n">
@@ -1356,77 +1368,26 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Sidoinkomst</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="n">
-        <v>2000</v>
-      </c>
-      <c r="C4" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="10">
-        <f>C4-B4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Bidrag / Studiestöd</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="10">
-        <f>C5-B5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Övrigt</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="10">
-        <f>C6-B6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>TOTALT</t>
         </is>
       </c>
-      <c r="B7" s="18">
-        <f>SUM(B2:B6)</f>
-        <v/>
-      </c>
-      <c r="C7" s="18">
-        <f>SUM(C2:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="18">
-        <f>SUM(D2:D6)</f>
+      <c r="B4" s="18">
+        <f>SUM(B2:B3)</f>
+        <v/>
+      </c>
+      <c r="C4" s="18">
+        <f>SUM(C2:C3)</f>
+        <v/>
+      </c>
+      <c r="D4" s="18">
+        <f>SUM(D2:D3)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D6">
+  <conditionalFormatting sqref="D2:D3">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1513,11 +1474,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
+      <c r="A2" s="13" t="n"/>
       <c r="B2" s="20" t="inlineStr">
         <is>
           <t>Boende</t>
@@ -1529,10 +1486,10 @@
         </is>
       </c>
       <c r="D2" s="10" t="n">
-        <v>12000</v>
+        <v>3914</v>
       </c>
       <c r="E2" s="10" t="n">
-        <v>12000</v>
+        <v>0</v>
       </c>
       <c r="F2" s="10">
         <f>IF(AND(D2=0,E2=0),"",D2-E2)</f>
@@ -1557,11 +1514,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>2026-04-02</t>
-        </is>
-      </c>
+      <c r="A3" s="13" t="n"/>
       <c r="B3" s="20" t="inlineStr">
         <is>
           <t>Mat</t>
@@ -1569,11 +1522,11 @@
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>Veckohandling</t>
+          <t>Matbudget</t>
         </is>
       </c>
       <c r="D3" s="10" t="n">
-        <v>1800</v>
+        <v>6200</v>
       </c>
       <c r="E3" s="10" t="n">
         <v>0</v>
@@ -1601,11 +1554,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>2026-04-03</t>
-        </is>
-      </c>
+      <c r="A4" s="13" t="n"/>
       <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Transport</t>
@@ -1613,14 +1562,14 @@
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>SL-kort</t>
+          <t>Diesel</t>
         </is>
       </c>
       <c r="D4" s="10" t="n">
-        <v>1020</v>
+        <v>2750</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>1020</v>
+        <v>0</v>
       </c>
       <c r="F4" s="10">
         <f>IF(AND(D4=0,E4=0),"",D4-E4)</f>
@@ -1645,23 +1594,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>2026-04-05</t>
-        </is>
-      </c>
+      <c r="A5" s="13" t="n"/>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>Prenumerationer</t>
+          <t>Transport</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>Spotify + Netflix</t>
+          <t>Underhåll bil/mc</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
-        <v>250</v>
+        <v>1000</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>0</v>
@@ -1690,10 +1635,22 @@
     </row>
     <row r="6">
       <c r="A6" s="13" t="n"/>
-      <c r="B6" s="20" t="n"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Bilskatt (5639 kr/år ÷ 12)</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>470</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F6" s="10">
         <f>IF(AND(D6=0,E6=0),"",D6-E6)</f>
         <v/>
@@ -1718,10 +1675,22 @@
     </row>
     <row r="7">
       <c r="A7" s="13" t="n"/>
-      <c r="B7" s="20" t="n"/>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Försäkring</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Bilförsäkring (416 kr/år ÷ 12)</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F7" s="10">
         <f>IF(AND(D7=0,E7=0),"",D7-E7)</f>
         <v/>
@@ -1746,10 +1715,22 @@
     </row>
     <row r="8">
       <c r="A8" s="13" t="n"/>
-      <c r="B8" s="20" t="n"/>
-      <c r="C8" s="20" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Försäkring</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>A-kassa</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>160</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F8" s="10">
         <f>IF(AND(D8=0,E8=0),"",D8-E8)</f>
         <v/>
@@ -1774,10 +1755,22 @@
     </row>
     <row r="9">
       <c r="A9" s="13" t="n"/>
-      <c r="B9" s="20" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Prenumerationer</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>129</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F9" s="10">
         <f>IF(AND(D9=0,E9=0),"",D9-E9)</f>
         <v/>
@@ -1802,10 +1795,22 @@
     </row>
     <row r="10">
       <c r="A10" s="13" t="n"/>
-      <c r="B10" s="20" t="n"/>
-      <c r="C10" s="20" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Prenumerationer</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F10" s="10">
         <f>IF(AND(D10=0,E10=0),"",D10-E10)</f>
         <v/>
@@ -1830,10 +1835,22 @@
     </row>
     <row r="11">
       <c r="A11" s="13" t="n"/>
-      <c r="B11" s="20" t="n"/>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Prenumerationer</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F11" s="10">
         <f>IF(AND(D11=0,E11=0),"",D11-E11)</f>
         <v/>
@@ -1858,10 +1875,22 @@
     </row>
     <row r="12">
       <c r="A12" s="13" t="n"/>
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>Prenumerationer</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>Soundcloud</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>75</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F12" s="10">
         <f>IF(AND(D12=0,E12=0),"",D12-E12)</f>
         <v/>
@@ -1873,10 +1902,22 @@
     </row>
     <row r="13">
       <c r="A13" s="13" t="n"/>
-      <c r="B13" s="20" t="n"/>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>Prenumerationer</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>Claude Max</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F13" s="10">
         <f>IF(AND(D13=0,E13=0),"",D13-E13)</f>
         <v/>
@@ -1888,10 +1929,22 @@
     </row>
     <row r="14">
       <c r="A14" s="13" t="n"/>
-      <c r="B14" s="20" t="n"/>
-      <c r="C14" s="20" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>Prenumerationer</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>Systeme.io</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>160</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F14" s="10">
         <f>IF(AND(D14=0,E14=0),"",D14-E14)</f>
         <v/>
@@ -1903,10 +1956,22 @@
     </row>
     <row r="15">
       <c r="A15" s="13" t="n"/>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Hälsa</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>Linser</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F15" s="10">
         <f>IF(AND(D15=0,E15=0),"",D15-E15)</f>
         <v/>
@@ -1918,10 +1983,22 @@
     </row>
     <row r="16">
       <c r="A16" s="13" t="n"/>
-      <c r="B16" s="20" t="n"/>
-      <c r="C16" s="20" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>Kläder</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>Kläder och övriga utgifter</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F16" s="10">
         <f>IF(AND(D16=0,E16=0),"",D16-E16)</f>
         <v/>
@@ -2718,17 +2795,17 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Buffert (3 mån utgifter)</t>
+          <t>Buffert</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
         <v>60000</v>
       </c>
       <c r="C2" s="10" t="n">
-        <v>5000</v>
+        <v>34000</v>
       </c>
       <c r="D2" s="10" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="E2" s="10">
         <f>IF(B2="","",MAX(0,B2-C2))</f>
@@ -2750,17 +2827,17 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Semesterresa</t>
+          <t>Snöskoter</t>
         </is>
       </c>
       <c r="B3" s="10" t="n">
-        <v>25000</v>
+        <v>40000</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="E3" s="10">
         <f>IF(B3="","",MAX(0,B3-C3))</f>
@@ -2780,20 +2857,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Ny dator</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="n">
-        <v>18000</v>
-      </c>
-      <c r="C4" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="10" t="n">
-        <v>1000</v>
-      </c>
+      <c r="A4" s="20" t="n"/>
+      <c r="B4" s="10" t="n"/>
+      <c r="C4" s="10" t="n"/>
+      <c r="D4" s="10" t="n"/>
       <c r="E4" s="10">
         <f>IF(B4="","",MAX(0,B4-C4))</f>
         <v/>
@@ -2812,20 +2879,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Pension – extra</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="n">
-        <v>100000</v>
-      </c>
-      <c r="C5" s="10" t="n">
-        <v>12000</v>
-      </c>
-      <c r="D5" s="10" t="n">
-        <v>1500</v>
-      </c>
+      <c r="A5" s="20" t="n"/>
+      <c r="B5" s="10" t="n"/>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n"/>
       <c r="E5" s="10">
         <f>IF(B5="","",MAX(0,B5-C5))</f>
         <v/>
@@ -2943,4 +3000,78 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Konto</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>Saldo (kr)</t>
+        </is>
+      </c>
+      <c r="C1" s="16" t="inlineStr">
+        <is>
+          <t>Anteckning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Sparkonto</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n">
+        <v>34000</v>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Behöver tas pengar härifrån denna månad</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Allkonto</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="n">
+        <v>2600</v>
+      </c>
+      <c r="C3" s="9" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>TOTALT</t>
+        </is>
+      </c>
+      <c r="B4" s="18">
+        <f>SUM(B2:B3)</f>
+        <v/>
+      </c>
+      <c r="C4" s="17" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix bilförsäkring to monthly and add missing recurring categories
Bilförsäkringen är 416 kr/månad (inte år) och budgeten saknade några
vanliga svenska hushållsutgifter. Lägger till tomma rader för el,
bredband, mobiltelefon och hemförsäkring som du själv fyller i.

https://claude.ai/code/session_01TGDrghwEeC6PfsKqYZFCU5
</commit_message>
<xml_diff>
--- a/Monthly_Budget_SEK.xlsx
+++ b/Monthly_Budget_SEK.xlsx
@@ -1517,16 +1517,16 @@
       <c r="A3" s="13" t="n"/>
       <c r="B3" s="20" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Räkningar</t>
         </is>
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>Matbudget</t>
+          <t>El (fyll i)</t>
         </is>
       </c>
       <c r="D3" s="10" t="n">
-        <v>6200</v>
+        <v>0</v>
       </c>
       <c r="E3" s="10" t="n">
         <v>0</v>
@@ -1557,16 +1557,16 @@
       <c r="A4" s="13" t="n"/>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>Räkningar</t>
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>Diesel</t>
+          <t>Bredband / internet (fyll i)</t>
         </is>
       </c>
       <c r="D4" s="10" t="n">
-        <v>2750</v>
+        <v>0</v>
       </c>
       <c r="E4" s="10" t="n">
         <v>0</v>
@@ -1597,16 +1597,16 @@
       <c r="A5" s="13" t="n"/>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>Räkningar</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>Underhåll bil/mc</t>
+          <t>Mobiltelefon (fyll i)</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>0</v>
@@ -1637,16 +1637,16 @@
       <c r="A6" s="13" t="n"/>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>Försäkring</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>Bilskatt (5639 kr/år ÷ 12)</t>
+          <t>Hemförsäkring (fyll i)</t>
         </is>
       </c>
       <c r="D6" s="10" t="n">
-        <v>470</v>
+        <v>0</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>0</v>
@@ -1677,16 +1677,16 @@
       <c r="A7" s="13" t="n"/>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>Försäkring</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>Bilförsäkring (416 kr/år ÷ 12)</t>
+          <t>Matbudget</t>
         </is>
       </c>
       <c r="D7" s="10" t="n">
-        <v>35</v>
+        <v>6200</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>0</v>
@@ -1717,16 +1717,16 @@
       <c r="A8" s="13" t="n"/>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Försäkring</t>
+          <t>Transport</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>A-kassa</t>
+          <t>Diesel</t>
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>160</v>
+        <v>2750</v>
       </c>
       <c r="E8" s="10" t="n">
         <v>0</v>
@@ -1757,16 +1757,16 @@
       <c r="A9" s="13" t="n"/>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>Prenumerationer</t>
+          <t>Transport</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>Spotify</t>
+          <t>Underhåll bil/mc</t>
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>129</v>
+        <v>1000</v>
       </c>
       <c r="E9" s="10" t="n">
         <v>0</v>
@@ -1797,16 +1797,16 @@
       <c r="A10" s="13" t="n"/>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Prenumerationer</t>
+          <t>Transport</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Bilskatt (5639 kr/år ÷ 12)</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>39</v>
+        <v>470</v>
       </c>
       <c r="E10" s="10" t="n">
         <v>0</v>
@@ -1837,16 +1837,16 @@
       <c r="A11" s="13" t="n"/>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>Prenumerationer</t>
+          <t>Försäkring</t>
         </is>
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Bilförsäkring</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>40</v>
+        <v>416</v>
       </c>
       <c r="E11" s="10" t="n">
         <v>0</v>
@@ -1877,16 +1877,16 @@
       <c r="A12" s="13" t="n"/>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Prenumerationer</t>
+          <t>Försäkring</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>Soundcloud</t>
+          <t>A-kassa</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>75</v>
+        <v>160</v>
       </c>
       <c r="E12" s="10" t="n">
         <v>0</v>
@@ -1909,11 +1909,11 @@
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
-          <t>Claude Max</t>
+          <t>Spotify</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>1300</v>
+        <v>129</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>0</v>
@@ -1936,11 +1936,11 @@
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>Systeme.io</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="D14" s="10" t="n">
-        <v>160</v>
+        <v>39</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>0</v>
@@ -1958,16 +1958,16 @@
       <c r="A15" s="13" t="n"/>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>Hälsa</t>
+          <t>Prenumerationer</t>
         </is>
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
-          <t>Linser</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="D15" s="10" t="n">
-        <v>500</v>
+        <v>40</v>
       </c>
       <c r="E15" s="10" t="n">
         <v>0</v>
@@ -1985,16 +1985,16 @@
       <c r="A16" s="13" t="n"/>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Kläder</t>
+          <t>Prenumerationer</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>Kläder och övriga utgifter</t>
+          <t>Soundcloud</t>
         </is>
       </c>
       <c r="D16" s="10" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>0</v>
@@ -2010,10 +2010,22 @@
     </row>
     <row r="17">
       <c r="A17" s="13" t="n"/>
-      <c r="B17" s="20" t="n"/>
-      <c r="C17" s="20" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>Prenumerationer</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>Claude Max</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F17" s="10">
         <f>IF(AND(D17=0,E17=0),"",D17-E17)</f>
         <v/>
@@ -2025,10 +2037,22 @@
     </row>
     <row r="18">
       <c r="A18" s="13" t="n"/>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>Prenumerationer</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Systeme.io</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>160</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F18" s="10">
         <f>IF(AND(D18=0,E18=0),"",D18-E18)</f>
         <v/>
@@ -2040,10 +2064,22 @@
     </row>
     <row r="19">
       <c r="A19" s="13" t="n"/>
-      <c r="B19" s="20" t="n"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>Hälsa</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>Linser</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F19" s="10">
         <f>IF(AND(D19=0,E19=0),"",D19-E19)</f>
         <v/>
@@ -2055,10 +2091,22 @@
     </row>
     <row r="20">
       <c r="A20" s="13" t="n"/>
-      <c r="B20" s="20" t="n"/>
-      <c r="C20" s="20" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>Kläder</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>Kläder och övriga utgifter</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="F20" s="10">
         <f>IF(AND(D20=0,E20=0),"",D20-E20)</f>
         <v/>

</xml_diff>

<commit_message>
Set monthly savings contributions (3 500 kr to each goal)
Jämn fördelning av månadssparandet: 3 500 kr till Buffert och 3 500 kr
till Snöskoter (totalt 7 000 kr/mån). Det lämnar ca 3 700 kr över för
kläder och oförutsett efter de fasta utgifterna.

https://claude.ai/code/session_01TGDrghwEeC6PfsKqYZFCU5
</commit_message>
<xml_diff>
--- a/Monthly_Budget_SEK.xlsx
+++ b/Monthly_Budget_SEK.xlsx
@@ -2853,7 +2853,7 @@
         <v>34000</v>
       </c>
       <c r="D2" s="10" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="E2" s="10">
         <f>IF(B2="","",MAX(0,B2-C2))</f>
@@ -2885,7 +2885,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="E3" s="10">
         <f>IF(B3="","",MAX(0,B3-C3))</f>

</xml_diff>

<commit_message>
Fill in el+bredband, mobilabonnemang and hemförsäkring
El + bredband 830 kr, mobilabonnemang 349 kr, hemförsäkring 100 kr.
Total fasta utgifter ökar till 18 432 kr/mån, vilket lämnar 2 408 kr
kvar för kläder och oförutsett efter att 7 000 kr satts av till sparmål.

https://claude.ai/code/session_01TGDrghwEeC6PfsKqYZFCU5
</commit_message>
<xml_diff>
--- a/Monthly_Budget_SEK.xlsx
+++ b/Monthly_Budget_SEK.xlsx
@@ -1522,11 +1522,11 @@
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>El (fyll i)</t>
+          <t>El + bredband</t>
         </is>
       </c>
       <c r="D3" s="10" t="n">
-        <v>0</v>
+        <v>830</v>
       </c>
       <c r="E3" s="10" t="n">
         <v>0</v>
@@ -1562,11 +1562,11 @@
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>Bredband / internet (fyll i)</t>
+          <t>Mobilabonnemang</t>
         </is>
       </c>
       <c r="D4" s="10" t="n">
-        <v>0</v>
+        <v>349</v>
       </c>
       <c r="E4" s="10" t="n">
         <v>0</v>
@@ -1597,16 +1597,16 @@
       <c r="A5" s="13" t="n"/>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>Räkningar</t>
+          <t>Försäkring</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>Mobiltelefon (fyll i)</t>
+          <t>Hemförsäkring</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>0</v>
@@ -1637,16 +1637,16 @@
       <c r="A6" s="13" t="n"/>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Försäkring</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>Hemförsäkring (fyll i)</t>
+          <t>Matbudget</t>
         </is>
       </c>
       <c r="D6" s="10" t="n">
-        <v>0</v>
+        <v>6200</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>0</v>
@@ -1677,16 +1677,16 @@
       <c r="A7" s="13" t="n"/>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Transport</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>Matbudget</t>
+          <t>Diesel</t>
         </is>
       </c>
       <c r="D7" s="10" t="n">
-        <v>6200</v>
+        <v>2750</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>0</v>
@@ -1722,11 +1722,11 @@
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>Diesel</t>
+          <t>Underhåll bil/mc</t>
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>2750</v>
+        <v>1000</v>
       </c>
       <c r="E8" s="10" t="n">
         <v>0</v>
@@ -1762,11 +1762,11 @@
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>Underhåll bil/mc</t>
+          <t>Bilskatt (5639 kr/år ÷ 12)</t>
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>1000</v>
+        <v>470</v>
       </c>
       <c r="E9" s="10" t="n">
         <v>0</v>
@@ -1797,16 +1797,16 @@
       <c r="A10" s="13" t="n"/>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>Försäkring</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>Bilskatt (5639 kr/år ÷ 12)</t>
+          <t>Bilförsäkring</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>470</v>
+        <v>416</v>
       </c>
       <c r="E10" s="10" t="n">
         <v>0</v>
@@ -1842,11 +1842,11 @@
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
-          <t>Bilförsäkring</t>
+          <t>A-kassa</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>416</v>
+        <v>160</v>
       </c>
       <c r="E11" s="10" t="n">
         <v>0</v>
@@ -1877,16 +1877,16 @@
       <c r="A12" s="13" t="n"/>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Försäkring</t>
+          <t>Prenumerationer</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>A-kassa</t>
+          <t>Spotify</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="E12" s="10" t="n">
         <v>0</v>
@@ -1909,11 +1909,11 @@
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
-          <t>Spotify</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>129</v>
+        <v>39</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>0</v>
@@ -1936,11 +1936,11 @@
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="D14" s="10" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>0</v>
@@ -1963,11 +1963,11 @@
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Soundcloud</t>
         </is>
       </c>
       <c r="D15" s="10" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="E15" s="10" t="n">
         <v>0</v>
@@ -1990,11 +1990,11 @@
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>Soundcloud</t>
+          <t>Claude Max</t>
         </is>
       </c>
       <c r="D16" s="10" t="n">
-        <v>75</v>
+        <v>1300</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>0</v>
@@ -2017,11 +2017,11 @@
       </c>
       <c r="C17" s="20" t="inlineStr">
         <is>
-          <t>Claude Max</t>
+          <t>Systeme.io</t>
         </is>
       </c>
       <c r="D17" s="10" t="n">
-        <v>1300</v>
+        <v>160</v>
       </c>
       <c r="E17" s="10" t="n">
         <v>0</v>
@@ -2039,16 +2039,16 @@
       <c r="A18" s="13" t="n"/>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Prenumerationer</t>
+          <t>Hälsa</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>Systeme.io</t>
+          <t>Linser</t>
         </is>
       </c>
       <c r="D18" s="10" t="n">
-        <v>160</v>
+        <v>500</v>
       </c>
       <c r="E18" s="10" t="n">
         <v>0</v>
@@ -2066,16 +2066,16 @@
       <c r="A19" s="13" t="n"/>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>Hälsa</t>
+          <t>Kläder</t>
         </is>
       </c>
       <c r="C19" s="20" t="inlineStr">
         <is>
-          <t>Linser</t>
+          <t>Kläder och övriga utgifter</t>
         </is>
       </c>
       <c r="D19" s="10" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="E19" s="10" t="n">
         <v>0</v>
@@ -2091,22 +2091,10 @@
     </row>
     <row r="20">
       <c r="A20" s="13" t="n"/>
-      <c r="B20" s="20" t="inlineStr">
-        <is>
-          <t>Kläder</t>
-        </is>
-      </c>
-      <c r="C20" s="20" t="inlineStr">
-        <is>
-          <t>Kläder och övriga utgifter</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="B20" s="20" t="n"/>
+      <c r="C20" s="20" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
       <c r="F20" s="10">
         <f>IF(AND(D20=0,E20=0),"",D20-E20)</f>
         <v/>

</xml_diff>

<commit_message>
Balansera budgeten: prioritera buffert och ge kläder en riktig budget
Sätter "Kläder och övriga utgifter" till 1 500 kr/mån i stället för 0,
och flyttar 1 500 kr av månadssparandet från snöskotern till bufferten
(5 000 kr buffert + 2 000 kr snöskoter). Bufferten blir då full på 6 mån
och du behöver inte dra ur sparkontot framöver. 908 kr lämnas okvarstad
som marginal för oförutsett.

https://claude.ai/code/session_01TGDrghwEeC6PfsKqYZFCU5
</commit_message>
<xml_diff>
--- a/Monthly_Budget_SEK.xlsx
+++ b/Monthly_Budget_SEK.xlsx
@@ -2075,7 +2075,7 @@
         </is>
       </c>
       <c r="D19" s="10" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="E19" s="10" t="n">
         <v>0</v>
@@ -2841,7 +2841,7 @@
         <v>34000</v>
       </c>
       <c r="D2" s="10" t="n">
-        <v>3500</v>
+        <v>5000</v>
       </c>
       <c r="E2" s="10">
         <f>IF(B2="","",MAX(0,B2-C2))</f>
@@ -2873,7 +2873,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="E3" s="10">
         <f>IF(B3="","",MAX(0,B3-C3))</f>

</xml_diff>